<commit_message>
Refresh 2026-08-06 Meta costs to final values and regenerate 08-07 report
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-08-07.xlsx
+++ b/data/reports/report-2026-08-07.xlsx
@@ -508,13 +508,13 @@
         <v>218974</v>
       </c>
       <c r="D2" t="n">
-        <v>441351</v>
+        <v>441601</v>
       </c>
       <c r="E2" t="n">
-        <v>137913</v>
+        <v>137663</v>
       </c>
       <c r="F2" t="n">
-        <v>17.28</v>
+        <v>17.25</v>
       </c>
       <c r="G2" t="n">
         <v>1.81</v>
@@ -526,7 +526,7 @@
         <v>27555</v>
       </c>
       <c r="J2" t="n">
-        <v>110358</v>
+        <v>110108</v>
       </c>
     </row>
     <row r="3">
@@ -542,13 +542,13 @@
         <v>761754</v>
       </c>
       <c r="D3" t="n">
-        <v>1466140</v>
+        <v>1466390</v>
       </c>
       <c r="E3" t="n">
-        <v>430094</v>
+        <v>429844</v>
       </c>
       <c r="F3" t="n">
-        <v>16.18</v>
+        <v>16.17</v>
       </c>
       <c r="G3" t="n">
         <v>1.81</v>
@@ -560,7 +560,7 @@
         <v>91754</v>
       </c>
       <c r="J3" t="n">
-        <v>338340</v>
+        <v>338090</v>
       </c>
     </row>
     <row r="4">
@@ -576,13 +576,13 @@
         <v>2192123</v>
       </c>
       <c r="D4" t="n">
-        <v>3598087</v>
+        <v>3598337</v>
       </c>
       <c r="E4" t="n">
-        <v>1738010</v>
+        <v>1737760</v>
       </c>
       <c r="F4" t="n">
-        <v>23.09</v>
+        <v>23.08</v>
       </c>
       <c r="G4" t="n">
         <v>2.09</v>
@@ -594,7 +594,7 @@
         <v>259874</v>
       </c>
       <c r="J4" t="n">
-        <v>1478136</v>
+        <v>1477886</v>
       </c>
     </row>
     <row r="5">
@@ -610,10 +610,10 @@
         <v>11292628</v>
       </c>
       <c r="D5" t="n">
-        <v>15347548</v>
+        <v>15347798</v>
       </c>
       <c r="E5" t="n">
-        <v>11276992</v>
+        <v>11276742</v>
       </c>
       <c r="F5" t="n">
         <v>29.74</v>
@@ -628,7 +628,7 @@
         <v>1308901</v>
       </c>
       <c r="J5" t="n">
-        <v>9968091</v>
+        <v>9967841</v>
       </c>
     </row>
   </sheetData>
@@ -758,10 +758,10 @@
         <v>252737</v>
       </c>
       <c r="D2" t="n">
-        <v>531381</v>
+        <v>531404</v>
       </c>
       <c r="E2" t="n">
-        <v>537839</v>
+        <v>537816</v>
       </c>
       <c r="F2" t="n">
         <v>2.49</v>
@@ -776,16 +776,16 @@
         <v>189448</v>
       </c>
       <c r="J2" t="n">
-        <v>73696</v>
+        <v>73673</v>
       </c>
       <c r="K2" t="n">
         <v>38.9</v>
       </c>
       <c r="L2" t="n">
-        <v>175396</v>
+        <v>175373</v>
       </c>
       <c r="M2" t="n">
-        <v>1802300</v>
+        <v>1802277</v>
       </c>
       <c r="N2" t="n">
         <v>336</v>
@@ -814,10 +814,10 @@
         <v>352920</v>
       </c>
       <c r="D3" t="n">
-        <v>434081</v>
+        <v>434095</v>
       </c>
       <c r="E3" t="n">
-        <v>173890</v>
+        <v>173876</v>
       </c>
       <c r="F3" t="n">
         <v>2.21</v>
@@ -832,16 +832,16 @@
         <v>60756</v>
       </c>
       <c r="J3" t="n">
-        <v>-7956</v>
+        <v>-7970</v>
       </c>
       <c r="K3" t="n">
         <v>-13.1</v>
       </c>
       <c r="L3" t="n">
-        <v>24552</v>
+        <v>24538</v>
       </c>
       <c r="M3" t="n">
-        <v>2181263</v>
+        <v>2181249</v>
       </c>
       <c r="N3" t="n">
         <v>204</v>
@@ -868,10 +868,10 @@
         <v>189873</v>
       </c>
       <c r="D4" t="n">
-        <v>385774</v>
+        <v>385790</v>
       </c>
       <c r="E4" t="n">
-        <v>223935</v>
+        <v>223919</v>
       </c>
       <c r="F4" t="n">
         <v>2.07</v>
@@ -886,16 +886,16 @@
         <v>62685</v>
       </c>
       <c r="J4" t="n">
-        <v>8701</v>
+        <v>8685</v>
       </c>
       <c r="K4" t="n">
         <v>13.9</v>
       </c>
       <c r="L4" t="n">
-        <v>73001</v>
+        <v>72985</v>
       </c>
       <c r="M4" t="n">
-        <v>1960089</v>
+        <v>1960073</v>
       </c>
       <c r="N4" t="n">
         <v>219</v>
@@ -922,10 +922,10 @@
         <v>197659</v>
       </c>
       <c r="D5" t="n">
-        <v>364608</v>
+        <v>364639</v>
       </c>
       <c r="E5" t="n">
-        <v>170042</v>
+        <v>170011</v>
       </c>
       <c r="F5" t="n">
         <v>2.01</v>
@@ -940,16 +940,16 @@
         <v>73704</v>
       </c>
       <c r="J5" t="n">
-        <v>17713</v>
+        <v>17682</v>
       </c>
       <c r="K5" t="n">
         <v>24</v>
       </c>
       <c r="L5" t="n">
-        <v>29015</v>
+        <v>28984</v>
       </c>
       <c r="M5" t="n">
-        <v>1765334</v>
+        <v>1765303</v>
       </c>
       <c r="N5" t="n">
         <v>151</v>
@@ -976,10 +976,10 @@
         <v>199326</v>
       </c>
       <c r="D6" t="n">
-        <v>224325</v>
+        <v>224355</v>
       </c>
       <c r="E6" t="n">
-        <v>115440</v>
+        <v>115410</v>
       </c>
       <c r="F6" t="n">
         <v>2.4</v>
@@ -994,16 +994,16 @@
         <v>46964</v>
       </c>
       <c r="J6" t="n">
-        <v>-19</v>
+        <v>-49</v>
       </c>
       <c r="K6" t="n">
-        <v>-0</v>
+        <v>-0.1</v>
       </c>
       <c r="L6" t="n">
-        <v>22255</v>
+        <v>22225</v>
       </c>
       <c r="M6" t="n">
-        <v>672967</v>
+        <v>672937</v>
       </c>
       <c r="N6" t="n">
         <v>139</v>
@@ -1030,10 +1030,10 @@
         <v>129591</v>
       </c>
       <c r="D7" t="n">
-        <v>226565</v>
+        <v>226572</v>
       </c>
       <c r="E7" t="n">
-        <v>126406</v>
+        <v>126399</v>
       </c>
       <c r="F7" t="n">
         <v>2.13</v>
@@ -1048,16 +1048,16 @@
         <v>54780</v>
       </c>
       <c r="J7" t="n">
-        <v>10410</v>
+        <v>10403</v>
       </c>
       <c r="K7" t="n">
         <v>19</v>
       </c>
       <c r="L7" t="n">
-        <v>13749</v>
+        <v>13742</v>
       </c>
       <c r="M7" t="n">
-        <v>789636</v>
+        <v>789629</v>
       </c>
       <c r="N7" t="n">
         <v>99</v>
@@ -1084,10 +1084,10 @@
         <v>179072</v>
       </c>
       <c r="D8" t="n">
-        <v>121299</v>
+        <v>121302</v>
       </c>
       <c r="E8" t="n">
-        <v>146349</v>
+        <v>146346</v>
       </c>
       <c r="F8" t="n">
         <v>3.68</v>
@@ -1102,16 +1102,16 @@
         <v>27920</v>
       </c>
       <c r="J8" t="n">
-        <v>-1958</v>
+        <v>-1961</v>
       </c>
       <c r="K8" t="n">
         <v>-7</v>
       </c>
       <c r="L8" t="n">
-        <v>34628</v>
+        <v>34625</v>
       </c>
       <c r="M8" t="n">
-        <v>287459</v>
+        <v>287456</v>
       </c>
       <c r="N8" t="n">
         <v>64</v>
@@ -1138,10 +1138,10 @@
         <v>142296</v>
       </c>
       <c r="D9" t="n">
-        <v>125676</v>
+        <v>125677</v>
       </c>
       <c r="E9" t="n">
-        <v>98307</v>
+        <v>98306</v>
       </c>
       <c r="F9" t="n">
         <v>2.91</v>
@@ -1156,16 +1156,16 @@
         <v>52788</v>
       </c>
       <c r="J9" t="n">
-        <v>17137</v>
+        <v>17136</v>
       </c>
       <c r="K9" t="n">
         <v>32.5</v>
       </c>
       <c r="L9" t="n">
-        <v>21631</v>
+        <v>21630</v>
       </c>
       <c r="M9" t="n">
-        <v>359884</v>
+        <v>359883</v>
       </c>
       <c r="N9" t="n">
         <v>77</v>
@@ -1192,10 +1192,10 @@
         <v>97804</v>
       </c>
       <c r="D10" t="n">
-        <v>147426</v>
+        <v>147428</v>
       </c>
       <c r="E10" t="n">
-        <v>40614</v>
+        <v>40612</v>
       </c>
       <c r="F10" t="n">
         <v>1.94</v>
@@ -1210,16 +1210,16 @@
         <v>5980</v>
       </c>
       <c r="J10" t="n">
-        <v>-8436</v>
+        <v>-8438</v>
       </c>
       <c r="K10" t="n">
         <v>-141.1</v>
       </c>
       <c r="L10" t="n">
-        <v>-6566</v>
+        <v>-6568</v>
       </c>
       <c r="M10" t="n">
-        <v>553670</v>
+        <v>553668</v>
       </c>
       <c r="N10" t="n">
         <v>49</v>
@@ -1246,10 +1246,10 @@
         <v>58938</v>
       </c>
       <c r="D11" t="n">
-        <v>150042</v>
+        <v>150057</v>
       </c>
       <c r="E11" t="n">
-        <v>48924</v>
+        <v>48909</v>
       </c>
       <c r="F11" t="n">
         <v>1.72</v>
@@ -1264,16 +1264,16 @@
         <v>27064</v>
       </c>
       <c r="J11" t="n">
-        <v>-3388</v>
+        <v>-3403</v>
       </c>
       <c r="K11" t="n">
-        <v>-12.5</v>
+        <v>-12.6</v>
       </c>
       <c r="L11" t="n">
-        <v>-6474</v>
+        <v>-6489</v>
       </c>
       <c r="M11" t="n">
-        <v>359729</v>
+        <v>359714</v>
       </c>
       <c r="N11" t="n">
         <v>66</v>
@@ -1300,10 +1300,10 @@
         <v>67374</v>
       </c>
       <c r="D12" t="n">
-        <v>63747</v>
+        <v>63748</v>
       </c>
       <c r="E12" t="n">
-        <v>92555</v>
+        <v>92554</v>
       </c>
       <c r="F12" t="n">
         <v>3.51</v>
@@ -1318,16 +1318,16 @@
         <v>63680</v>
       </c>
       <c r="J12" t="n">
-        <v>27389</v>
+        <v>27388</v>
       </c>
       <c r="K12" t="n">
         <v>43</v>
       </c>
       <c r="L12" t="n">
-        <v>73015</v>
+        <v>73014</v>
       </c>
       <c r="M12" t="n">
-        <v>92555</v>
+        <v>92554</v>
       </c>
       <c r="N12" t="n">
         <v>57</v>
@@ -1466,10 +1466,10 @@
         <v>29008</v>
       </c>
       <c r="D15" t="n">
-        <v>117597</v>
+        <v>117602</v>
       </c>
       <c r="E15" t="n">
-        <v>-2728</v>
+        <v>-2733</v>
       </c>
       <c r="F15" t="n">
         <v>1.22</v>
@@ -1484,22 +1484,22 @@
         <v>26069</v>
       </c>
       <c r="J15" t="n">
-        <v>6653</v>
+        <v>6648</v>
       </c>
       <c r="K15" t="n">
         <v>25.5</v>
       </c>
       <c r="L15" t="n">
-        <v>-3212</v>
+        <v>-3217</v>
       </c>
       <c r="M15" t="n">
-        <v>253986</v>
+        <v>253981</v>
       </c>
       <c r="N15" t="n">
         <v>37</v>
       </c>
       <c r="O15" t="n">
-        <v>12500</v>
+        <v>8000</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
@@ -1520,10 +1520,10 @@
         <v>47061</v>
       </c>
       <c r="D16" t="n">
-        <v>72428</v>
+        <v>72429</v>
       </c>
       <c r="E16" t="n">
-        <v>14971</v>
+        <v>14970</v>
       </c>
       <c r="F16" t="n">
         <v>1.86</v>
@@ -1538,16 +1538,16 @@
         <v>14940</v>
       </c>
       <c r="J16" t="n">
-        <v>-530</v>
+        <v>-531</v>
       </c>
       <c r="K16" t="n">
-        <v>-3.5</v>
+        <v>-3.6</v>
       </c>
       <c r="L16" t="n">
-        <v>3997</v>
+        <v>3996</v>
       </c>
       <c r="M16" t="n">
-        <v>88445</v>
+        <v>88444</v>
       </c>
       <c r="N16" t="n">
         <v>27</v>
@@ -1688,13 +1688,13 @@
         <v>23543</v>
       </c>
       <c r="D19" t="n">
-        <v>33853</v>
+        <v>33871</v>
       </c>
       <c r="E19" t="n">
-        <v>22344</v>
+        <v>22326</v>
       </c>
       <c r="F19" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
       <c r="G19" t="n">
         <v>1.42</v>
@@ -1706,16 +1706,16 @@
         <v>23920</v>
       </c>
       <c r="J19" t="n">
-        <v>7665</v>
+        <v>7647</v>
       </c>
       <c r="K19" t="n">
         <v>32</v>
       </c>
       <c r="L19" t="n">
-        <v>16175</v>
+        <v>16157</v>
       </c>
       <c r="M19" t="n">
-        <v>22344</v>
+        <v>22326</v>
       </c>
       <c r="N19" t="n">
         <v>13</v>
@@ -1742,10 +1742,10 @@
         <v>15648</v>
       </c>
       <c r="D20" t="n">
-        <v>34638</v>
+        <v>34641</v>
       </c>
       <c r="E20" t="n">
-        <v>6486</v>
+        <v>6483</v>
       </c>
       <c r="F20" t="n">
         <v>1.64</v>
@@ -1760,16 +1760,16 @@
         <v>13944</v>
       </c>
       <c r="J20" t="n">
-        <v>4283</v>
+        <v>4280</v>
       </c>
       <c r="K20" t="n">
         <v>30.7</v>
       </c>
       <c r="L20" t="n">
-        <v>8890</v>
+        <v>8887</v>
       </c>
       <c r="M20" t="n">
-        <v>53242</v>
+        <v>53239</v>
       </c>
       <c r="N20" t="n">
         <v>12</v>
@@ -2282,10 +2282,10 @@
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>6400</v>
+        <v>6413</v>
       </c>
       <c r="E29" t="n">
-        <v>-1420</v>
+        <v>-1433</v>
       </c>
       <c r="F29" t="n">
         <v>0.78</v>
@@ -2300,16 +2300,16 @@
         <v>4980</v>
       </c>
       <c r="J29" t="n">
-        <v>-1420</v>
+        <v>-1433</v>
       </c>
       <c r="K29" t="n">
-        <v>-28.5</v>
+        <v>-28.8</v>
       </c>
       <c r="L29" t="n">
-        <v>-1420</v>
+        <v>-1433</v>
       </c>
       <c r="M29" t="n">
-        <v>-1420</v>
+        <v>-1433</v>
       </c>
       <c r="N29" t="n">
         <v>1</v>
@@ -2340,7 +2340,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>190576</v>
+        <v>190643</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -2827,16 +2827,16 @@
         <v>798238</v>
       </c>
       <c r="D15" t="n">
-        <v>441351</v>
+        <v>441601</v>
       </c>
       <c r="E15" t="n">
-        <v>138093</v>
+        <v>137843</v>
       </c>
       <c r="F15" t="n">
-        <v>17.3</v>
+        <v>17.27</v>
       </c>
       <c r="G15" t="n">
-        <v>143516</v>
+        <v>143433</v>
       </c>
     </row>
   </sheetData>

</xml_diff>